<commit_message>
update data view and visualization
</commit_message>
<xml_diff>
--- a/analysis/dataview/binary-tree-CoT.xlsx
+++ b/analysis/dataview/binary-tree-CoT.xlsx
@@ -536,10 +536,10 @@
         <v>10</v>
       </c>
       <c r="B2">
-        <v>76.81333333333333</v>
+        <v>49.30458333333333</v>
       </c>
       <c r="C2">
-        <v>17.41993702046886</v>
+        <v>26.50397623641743</v>
       </c>
       <c r="D2">
         <v>24</v>
@@ -550,10 +550,10 @@
         <v>11</v>
       </c>
       <c r="B3">
-        <v>14.68</v>
+        <v>29.30208333333333</v>
       </c>
       <c r="C3">
-        <v>20.06330979674092</v>
+        <v>28.65332395607679</v>
       </c>
       <c r="D3">
         <v>24</v>
@@ -564,10 +564,10 @@
         <v>12</v>
       </c>
       <c r="B4">
-        <v>4.032083333333333</v>
+        <v>5.74875</v>
       </c>
       <c r="C4">
-        <v>7.428896564542185</v>
+        <v>9.818091248347082</v>
       </c>
       <c r="D4">
         <v>24</v>
@@ -578,10 +578,10 @@
         <v>13</v>
       </c>
       <c r="B5">
-        <v>24.44</v>
+        <v>36.74666666666666</v>
       </c>
       <c r="C5">
-        <v>26.68778698043439</v>
+        <v>33.40006595498132</v>
       </c>
       <c r="D5">
         <v>24</v>
@@ -592,10 +592,10 @@
         <v>14</v>
       </c>
       <c r="B6">
-        <v>27.06458333333333</v>
+        <v>40.49</v>
       </c>
       <c r="C6">
-        <v>29.15025005175273</v>
+        <v>34.19243941346505</v>
       </c>
       <c r="D6">
         <v>24</v>
@@ -644,10 +644,10 @@
         <v>16</v>
       </c>
       <c r="B2">
-        <v>33.90555555555555</v>
+        <v>34.16277777777778</v>
       </c>
       <c r="C2">
-        <v>33.40261172587476</v>
+        <v>32.8729325798692</v>
       </c>
       <c r="D2">
         <v>72</v>
@@ -658,10 +658,10 @@
         <v>17</v>
       </c>
       <c r="B3">
-        <v>36.31069444444444</v>
+        <v>40.9075</v>
       </c>
       <c r="C3">
-        <v>34.31167564294184</v>
+        <v>30.95816471750315</v>
       </c>
       <c r="D3">
         <v>72</v>
@@ -696,10 +696,10 @@
         <v>18</v>
       </c>
       <c r="B2">
-        <v>52.77770833333333</v>
+        <v>62.75979166666666</v>
       </c>
       <c r="C2">
-        <v>31.36111776392037</v>
+        <v>25.83347502506327</v>
       </c>
       <c r="D2">
         <v>48</v>
@@ -710,10 +710,10 @@
         <v>19</v>
       </c>
       <c r="B3">
-        <v>20.83395833333333</v>
+        <v>14.81520833333333</v>
       </c>
       <c r="C3">
-        <v>29.89561020501408</v>
+        <v>22.02411907959702</v>
       </c>
       <c r="D3">
         <v>48</v>
@@ -724,10 +724,10 @@
         <v>20</v>
       </c>
       <c r="B4">
-        <v>31.71270833333334</v>
+        <v>35.03041666666667</v>
       </c>
       <c r="C4">
-        <v>32.44037107505999</v>
+        <v>27.91516120954006</v>
       </c>
       <c r="D4">
         <v>48</v>
@@ -762,10 +762,10 @@
         <v>21</v>
       </c>
       <c r="B2">
-        <v>37.75083333333333</v>
+        <v>38.50263888888889</v>
       </c>
       <c r="C2">
-        <v>34.36420094135797</v>
+        <v>33.09207364322471</v>
       </c>
       <c r="D2">
         <v>72</v>
@@ -776,10 +776,10 @@
         <v>22</v>
       </c>
       <c r="B3">
-        <v>32.46541666666667</v>
+        <v>36.56763888888889</v>
       </c>
       <c r="C3">
-        <v>33.17974967591434</v>
+        <v>31.06637798047125</v>
       </c>
       <c r="D3">
         <v>72</v>
@@ -814,10 +814,10 @@
         <v>23</v>
       </c>
       <c r="B2">
-        <v>42.25208333333333</v>
+        <v>42.00736111111112</v>
       </c>
       <c r="C2">
-        <v>34.59927125901541</v>
+        <v>32.64889545801397</v>
       </c>
       <c r="D2">
         <v>72</v>
@@ -828,10 +828,10 @@
         <v>24</v>
       </c>
       <c r="B3">
-        <v>27.96416666666667</v>
+        <v>33.06291666666667</v>
       </c>
       <c r="C3">
-        <v>31.54899599973903</v>
+        <v>30.91259192077822</v>
       </c>
       <c r="D3">
         <v>72</v>

</xml_diff>